<commit_message>
Perform some excel function
</commit_message>
<xml_diff>
--- a/population.csv.xlsx
+++ b/population.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Indian Population Data Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5ED63F8-AA14-4807-BE25-B77AE7D423CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7702198-624F-4507-9079-0E8E6F0779C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
   </bookViews>
   <sheets>
     <sheet name="population" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId4"/>
-    <pivotCache cacheId="2" r:id="rId5"/>
+    <pivotCache cacheId="3" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="97">
   <si>
     <t>Rank</t>
   </si>
@@ -1322,7 +1322,43 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Females" numFmtId="3">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="31350" maxValue="95331831"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="31350" maxValue="95331831" count="35">
+        <n v="95331831"/>
+        <n v="54131277"/>
+        <n v="49821295"/>
+        <n v="44467088"/>
+        <n v="42138631"/>
+        <n v="35014503"/>
+        <n v="36009055"/>
+        <n v="32997440"/>
+        <n v="30128640"/>
+        <n v="28948432"/>
+        <n v="20762082"/>
+        <n v="17378649"/>
+        <n v="16057819"/>
+        <n v="15266133"/>
+        <n v="13103873"/>
+        <n v="12712303"/>
+        <n v="11856728"/>
+        <n v="7800615"/>
+        <n v="5900640"/>
+        <n v="4948519"/>
+        <n v="3382729"/>
+        <n v="1799541"/>
+        <n v="1475057"/>
+        <n v="1280219"/>
+        <n v="953853"/>
+        <n v="719405"/>
+        <n v="669815"/>
+        <n v="635442"/>
+        <n v="541867"/>
+        <n v="474787"/>
+        <n v="287507"/>
+        <n v="177710"/>
+        <n v="149949"/>
+        <n v="92946"/>
+        <n v="31350"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Gender Ratio" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="618" maxValue="1084" count="33">
@@ -2204,7 +2240,7 @@
     <n v="199812341"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="95331831"/>
+    <x v="0"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -2220,7 +2256,7 @@
     <n v="112374333"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="54131277"/>
+    <x v="1"/>
     <x v="1"/>
     <x v="1"/>
     <x v="1"/>
@@ -2236,7 +2272,7 @@
     <n v="104099452"/>
     <x v="2"/>
     <x v="2"/>
-    <n v="49821295"/>
+    <x v="2"/>
     <x v="2"/>
     <x v="2"/>
     <x v="2"/>
@@ -2252,7 +2288,7 @@
     <n v="91276115"/>
     <x v="3"/>
     <x v="3"/>
-    <n v="44467088"/>
+    <x v="3"/>
     <x v="3"/>
     <x v="3"/>
     <x v="3"/>
@@ -2268,7 +2304,7 @@
     <n v="84580777"/>
     <x v="4"/>
     <x v="4"/>
-    <n v="42138631"/>
+    <x v="4"/>
     <x v="4"/>
     <x v="4"/>
     <x v="4"/>
@@ -2284,7 +2320,7 @@
     <n v="72626809"/>
     <x v="5"/>
     <x v="5"/>
-    <n v="35014503"/>
+    <x v="5"/>
     <x v="5"/>
     <x v="5"/>
     <x v="5"/>
@@ -2300,7 +2336,7 @@
     <n v="72147030"/>
     <x v="6"/>
     <x v="6"/>
-    <n v="36009055"/>
+    <x v="6"/>
     <x v="6"/>
     <x v="6"/>
     <x v="6"/>
@@ -2316,7 +2352,7 @@
     <n v="68548437"/>
     <x v="7"/>
     <x v="7"/>
-    <n v="32997440"/>
+    <x v="7"/>
     <x v="7"/>
     <x v="7"/>
     <x v="7"/>
@@ -2332,7 +2368,7 @@
     <n v="61095297"/>
     <x v="8"/>
     <x v="8"/>
-    <n v="30128640"/>
+    <x v="8"/>
     <x v="8"/>
     <x v="8"/>
     <x v="8"/>
@@ -2348,7 +2384,7 @@
     <n v="60439692"/>
     <x v="9"/>
     <x v="9"/>
-    <n v="28948432"/>
+    <x v="9"/>
     <x v="9"/>
     <x v="9"/>
     <x v="9"/>
@@ -2364,7 +2400,7 @@
     <n v="41974218"/>
     <x v="10"/>
     <x v="10"/>
-    <n v="20762082"/>
+    <x v="10"/>
     <x v="10"/>
     <x v="10"/>
     <x v="10"/>
@@ -2380,7 +2416,7 @@
     <n v="33406061"/>
     <x v="11"/>
     <x v="11"/>
-    <n v="17378649"/>
+    <x v="11"/>
     <x v="11"/>
     <x v="11"/>
     <x v="11"/>
@@ -2396,7 +2432,7 @@
     <n v="32988134"/>
     <x v="12"/>
     <x v="12"/>
-    <n v="16057819"/>
+    <x v="12"/>
     <x v="12"/>
     <x v="12"/>
     <x v="12"/>
@@ -2412,7 +2448,7 @@
     <n v="31205576"/>
     <x v="13"/>
     <x v="13"/>
-    <n v="15266133"/>
+    <x v="13"/>
     <x v="13"/>
     <x v="13"/>
     <x v="13"/>
@@ -2428,7 +2464,7 @@
     <n v="27743338"/>
     <x v="14"/>
     <x v="14"/>
-    <n v="13103873"/>
+    <x v="14"/>
     <x v="14"/>
     <x v="14"/>
     <x v="14"/>
@@ -2444,7 +2480,7 @@
     <n v="25545198"/>
     <x v="15"/>
     <x v="15"/>
-    <n v="12712303"/>
+    <x v="15"/>
     <x v="15"/>
     <x v="15"/>
     <x v="15"/>
@@ -2460,7 +2496,7 @@
     <n v="25351462"/>
     <x v="16"/>
     <x v="16"/>
-    <n v="11856728"/>
+    <x v="16"/>
     <x v="16"/>
     <x v="16"/>
     <x v="16"/>
@@ -2476,7 +2512,7 @@
     <n v="16787941"/>
     <x v="17"/>
     <x v="17"/>
-    <n v="7800615"/>
+    <x v="17"/>
     <x v="17"/>
     <x v="17"/>
     <x v="17"/>
@@ -2492,7 +2528,7 @@
     <n v="12541302"/>
     <x v="18"/>
     <x v="18"/>
-    <n v="5900640"/>
+    <x v="18"/>
     <x v="18"/>
     <x v="18"/>
     <x v="18"/>
@@ -2508,7 +2544,7 @@
     <n v="10086292"/>
     <x v="19"/>
     <x v="19"/>
-    <n v="4948519"/>
+    <x v="19"/>
     <x v="19"/>
     <x v="19"/>
     <x v="19"/>
@@ -2524,7 +2560,7 @@
     <n v="6864602"/>
     <x v="20"/>
     <x v="20"/>
-    <n v="3382729"/>
+    <x v="20"/>
     <x v="20"/>
     <x v="20"/>
     <x v="20"/>
@@ -2540,7 +2576,7 @@
     <n v="3673917"/>
     <x v="21"/>
     <x v="21"/>
-    <n v="1799541"/>
+    <x v="21"/>
     <x v="21"/>
     <x v="21"/>
     <x v="21"/>
@@ -2556,7 +2592,7 @@
     <n v="2966889"/>
     <x v="22"/>
     <x v="22"/>
-    <n v="1475057"/>
+    <x v="22"/>
     <x v="22"/>
     <x v="22"/>
     <x v="22"/>
@@ -2572,7 +2608,7 @@
     <n v="2721756"/>
     <x v="23"/>
     <x v="23"/>
-    <n v="1280219"/>
+    <x v="23"/>
     <x v="23"/>
     <x v="23"/>
     <x v="23"/>
@@ -2588,7 +2624,7 @@
     <n v="1978502"/>
     <x v="24"/>
     <x v="24"/>
-    <n v="953853"/>
+    <x v="24"/>
     <x v="5"/>
     <x v="24"/>
     <x v="24"/>
@@ -2604,7 +2640,7 @@
     <n v="1458545"/>
     <x v="25"/>
     <x v="25"/>
-    <n v="719405"/>
+    <x v="25"/>
     <x v="8"/>
     <x v="25"/>
     <x v="25"/>
@@ -2620,7 +2656,7 @@
     <n v="1383727"/>
     <x v="26"/>
     <x v="26"/>
-    <n v="669815"/>
+    <x v="26"/>
     <x v="24"/>
     <x v="26"/>
     <x v="26"/>
@@ -2636,7 +2672,7 @@
     <n v="1247953"/>
     <x v="27"/>
     <x v="27"/>
-    <n v="635442"/>
+    <x v="27"/>
     <x v="25"/>
     <x v="27"/>
     <x v="27"/>
@@ -2652,7 +2688,7 @@
     <n v="1097206"/>
     <x v="28"/>
     <x v="28"/>
-    <n v="541867"/>
+    <x v="28"/>
     <x v="26"/>
     <x v="28"/>
     <x v="28"/>
@@ -2668,7 +2704,7 @@
     <n v="1055450"/>
     <x v="28"/>
     <x v="29"/>
-    <n v="474787"/>
+    <x v="29"/>
     <x v="27"/>
     <x v="29"/>
     <x v="29"/>
@@ -2684,7 +2720,7 @@
     <n v="610577"/>
     <x v="29"/>
     <x v="30"/>
-    <n v="287507"/>
+    <x v="30"/>
     <x v="28"/>
     <x v="30"/>
     <x v="30"/>
@@ -2700,7 +2736,7 @@
     <n v="380581"/>
     <x v="30"/>
     <x v="31"/>
-    <n v="177710"/>
+    <x v="31"/>
     <x v="29"/>
     <x v="31"/>
     <x v="31"/>
@@ -2716,7 +2752,7 @@
     <n v="343709"/>
     <x v="30"/>
     <x v="32"/>
-    <n v="149949"/>
+    <x v="32"/>
     <x v="30"/>
     <x v="32"/>
     <x v="32"/>
@@ -2732,7 +2768,7 @@
     <n v="243247"/>
     <x v="31"/>
     <x v="33"/>
-    <n v="92946"/>
+    <x v="33"/>
     <x v="31"/>
     <x v="33"/>
     <x v="33"/>
@@ -2748,7 +2784,7 @@
     <n v="64473"/>
     <x v="32"/>
     <x v="34"/>
-    <n v="31350"/>
+    <x v="34"/>
     <x v="32"/>
     <x v="34"/>
     <x v="34"/>
@@ -2761,8 +2797,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="M5:N76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{62D21C4D-F7A7-4C69-9E5C-A505D3EFBF2C}" name="PivotTable5" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="P5:Q41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -2805,346 +2841,166 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="34">
-        <item x="20"/>
-        <item x="27"/>
-        <item x="8"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item x="31"/>
-        <item x="18"/>
-        <item x="16"/>
-        <item x="13"/>
-        <item x="9"/>
-        <item x="28"/>
-        <item x="4"/>
-        <item x="22"/>
-        <item x="25"/>
-        <item x="7"/>
-        <item x="17"/>
-        <item x="32"/>
-        <item x="23"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="24"/>
-        <item x="2"/>
-        <item x="26"/>
-        <item x="29"/>
-        <item x="15"/>
-        <item x="12"/>
-        <item x="21"/>
-        <item x="19"/>
-        <item x="30"/>
-        <item x="11"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField numFmtId="3" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
+    <pivotField axis="axisPage" numFmtId="3" showAll="0">
       <items count="36">
         <item x="34"/>
         <item x="33"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="30"/>
         <item x="29"/>
+        <item x="28"/>
         <item x="27"/>
-        <item x="32"/>
-        <item x="17"/>
+        <item x="26"/>
         <item x="25"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="21"/>
         <item x="24"/>
-        <item x="28"/>
         <item x="23"/>
         <item x="22"/>
-        <item x="11"/>
+        <item x="21"/>
+        <item x="20"/>
+        <item x="19"/>
+        <item x="18"/>
+        <item x="17"/>
         <item x="16"/>
+        <item x="15"/>
         <item x="14"/>
-        <item x="19"/>
-        <item x="20"/>
         <item x="13"/>
         <item x="12"/>
-        <item x="26"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="4"/>
         <item x="3"/>
         <item x="2"/>
-        <item x="6"/>
-        <item x="15"/>
-        <item x="10"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="18"/>
+        <item x="1"/>
         <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="34">
-        <item x="24"/>
-        <item x="29"/>
-        <item x="26"/>
-        <item x="17"/>
-        <item x="28"/>
-        <item x="22"/>
-        <item x="21"/>
-        <item x="18"/>
-        <item x="20"/>
-        <item x="14"/>
-        <item x="7"/>
-        <item x="5"/>
-        <item x="9"/>
-        <item x="4"/>
-        <item x="8"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="23"/>
-        <item x="12"/>
-        <item x="11"/>
-        <item x="13"/>
-        <item x="6"/>
-        <item x="15"/>
-        <item x="30"/>
-        <item x="0"/>
-        <item x="10"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="32"/>
-        <item x="31"/>
-        <item x="25"/>
-        <item x="27"/>
-        <item x="16"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
-  <rowFields count="2">
+  <rowFields count="1">
     <field x="1"/>
-    <field x="2"/>
   </rowFields>
-  <rowItems count="71">
+  <rowItems count="36">
     <i>
       <x/>
     </i>
-    <i r="1">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
       <x v="26"/>
     </i>
     <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
       <x v="27"/>
     </i>
     <i>
-      <x v="7"/>
-    </i>
-    <i r="1">
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
       <x v="31"/>
     </i>
     <i>
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i r="1">
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i r="1">
       <x v="32"/>
     </i>
     <i>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i r="1">
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i r="1">
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i r="1">
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i r="1">
-      <x v="21"/>
-    </i>
-    <i>
       <x v="33"/>
     </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
     <i>
       <x v="34"/>
-    </i>
-    <i r="1">
-      <x v="20"/>
     </i>
     <i t="grand">
       <x/>
@@ -3154,10 +3010,10 @@
     <i/>
   </colItems>
   <pageFields count="1">
-    <pageField fld="11" hier="-1"/>
+    <pageField fld="6" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Sum of % of Total Population" fld="4" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0" numFmtId="3"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3172,7 +3028,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:K39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -3441,7 +3297,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:G41" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0">
@@ -4082,6 +3938,417 @@
   </pageFields>
   <dataFields count="1">
     <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="M5:N76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="36">
+        <item x="31"/>
+        <item x="4"/>
+        <item x="26"/>
+        <item x="13"/>
+        <item x="2"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="9"/>
+        <item x="16"/>
+        <item x="20"/>
+        <item x="18"/>
+        <item x="12"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="34"/>
+        <item x="5"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="28"/>
+        <item x="24"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="30"/>
+        <item x="6"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="34">
+        <item x="20"/>
+        <item x="27"/>
+        <item x="8"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item x="31"/>
+        <item x="18"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="9"/>
+        <item x="28"/>
+        <item x="4"/>
+        <item x="22"/>
+        <item x="25"/>
+        <item x="7"/>
+        <item x="17"/>
+        <item x="32"/>
+        <item x="23"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="24"/>
+        <item x="2"/>
+        <item x="26"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="12"/>
+        <item x="21"/>
+        <item x="19"/>
+        <item x="30"/>
+        <item x="11"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="36">
+        <item x="34"/>
+        <item x="33"/>
+        <item x="29"/>
+        <item x="27"/>
+        <item x="32"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="21"/>
+        <item x="24"/>
+        <item x="28"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="14"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="26"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="6"/>
+        <item x="15"/>
+        <item x="10"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="18"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="34">
+        <item x="24"/>
+        <item x="29"/>
+        <item x="26"/>
+        <item x="17"/>
+        <item x="28"/>
+        <item x="22"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="20"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="12"/>
+        <item x="11"/>
+        <item x="13"/>
+        <item x="6"/>
+        <item x="15"/>
+        <item x="30"/>
+        <item x="0"/>
+        <item x="10"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="25"/>
+        <item x="27"/>
+        <item x="16"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="71">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i r="1">
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i r="1">
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i r="1">
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i r="1">
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i r="1">
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i r="1">
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i r="1">
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i r="1">
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i r="1">
+      <x v="20"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="11" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Sum of % of Total Population" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -6464,6 +6731,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
@@ -6476,12 +6749,6 @@
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6490,7 +6757,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881F210B-A9CA-4D54-9D0F-4913621E3B09}">
-  <dimension ref="A2:N76"/>
+  <dimension ref="A2:Q76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
@@ -6506,40 +6773,13 @@
     <col min="13" max="13" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="24.5546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="34" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="6" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="11" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="7" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="50" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E2" s="8" t="s">
         <v>8</v>
       </c>
@@ -6547,7 +6787,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
@@ -6572,8 +6812,14 @@
       <c r="N3" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>88</v>
       </c>
@@ -6604,8 +6850,14 @@
       <c r="N5" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P5" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>70</v>
       </c>
@@ -6637,8 +6889,14 @@
       <c r="N6">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P6" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q6" s="10">
+        <v>244411</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>72</v>
       </c>
@@ -6670,8 +6928,14 @@
       <c r="N7">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P7" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q7" s="10">
+        <v>56361702</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>35</v>
       </c>
@@ -6703,8 +6967,14 @@
       <c r="N8">
         <v>6.99</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P8" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q8" s="10">
+        <v>1069165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>76</v>
       </c>
@@ -6736,8 +7006,14 @@
       <c r="N9">
         <v>6.99</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P9" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" s="10">
+        <v>26780526</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>41</v>
       </c>
@@ -6769,8 +7045,14 @@
       <c r="N10">
         <v>0.11</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q10" s="10">
+        <v>92075028</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>48</v>
       </c>
@@ -6802,8 +7084,14 @@
       <c r="N11">
         <v>0.11</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P11" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q11" s="10">
+        <v>29004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>89</v>
       </c>
@@ -6835,8 +7123,14 @@
       <c r="N12">
         <v>2.58</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q12" s="10">
+        <v>19603658</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E13" s="9" t="s">
         <v>72</v>
       </c>
@@ -6862,8 +7156,14 @@
       <c r="N13">
         <v>2.58</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q13" s="10">
+        <v>183024</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E14" s="9" t="s">
         <v>74</v>
       </c>
@@ -6889,8 +7189,14 @@
       <c r="N14">
         <v>8.6</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P14" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q14" s="10">
+        <v>60331</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E15" s="9" t="s">
         <v>46</v>
       </c>
@@ -6916,8 +7222,14 @@
       <c r="N15">
         <v>8.6</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P15" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q15" s="10">
+        <v>944727</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E16" s="9" t="s">
         <v>60</v>
       </c>
@@ -6943,8 +7255,14 @@
       <c r="N16">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="17" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P16" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q16" s="10">
+        <v>551414</v>
+      </c>
+    </row>
+    <row r="17" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
         <v>31</v>
       </c>
@@ -6970,8 +7288,14 @@
       <c r="N17">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="18" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P17" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q17" s="10">
+        <v>34670817</v>
+      </c>
+    </row>
+    <row r="18" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E18" s="9" t="s">
         <v>45</v>
       </c>
@@ -6997,8 +7321,14 @@
       <c r="N18">
         <v>2.11</v>
       </c>
-    </row>
-    <row r="19" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P18" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q18" s="10">
+        <v>16531493</v>
+      </c>
+    </row>
+    <row r="19" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E19" s="9" t="s">
         <v>50</v>
       </c>
@@ -7024,8 +7354,14 @@
       <c r="N19">
         <v>2.11</v>
       </c>
-    </row>
-    <row r="20" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P19" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q19" s="10">
+        <v>6167805</v>
+      </c>
+    </row>
+    <row r="20" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
         <v>47</v>
       </c>
@@ -7051,8 +7387,14 @@
       <c r="N20">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="21" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P20" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q20" s="10">
+        <v>9134820</v>
+      </c>
+    </row>
+    <row r="21" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E21" s="9" t="s">
         <v>37</v>
       </c>
@@ -7078,8 +7420,14 @@
       <c r="N21">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="22" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P21" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q21" s="10">
+        <v>25036946</v>
+      </c>
+    </row>
+    <row r="22" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E22" s="9" t="s">
         <v>29</v>
       </c>
@@ -7105,8 +7453,14 @@
       <c r="N22">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="23" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P22" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q22" s="10">
+        <v>37552529</v>
+      </c>
+    </row>
+    <row r="23" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E23" s="9" t="s">
         <v>35</v>
       </c>
@@ -7132,8 +7486,14 @@
       <c r="N23">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="24" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P23" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q23" s="10">
+        <v>17445506</v>
+      </c>
+    </row>
+    <row r="24" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E24" s="9" t="s">
         <v>76</v>
       </c>
@@ -7159,8 +7519,14 @@
       <c r="N24">
         <v>1.39</v>
       </c>
-    </row>
-    <row r="25" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P24" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="10">
+        <v>14121</v>
+      </c>
+    </row>
+    <row r="25" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E25" s="9" t="s">
         <v>23</v>
       </c>
@@ -7186,8 +7552,14 @@
       <c r="N25">
         <v>1.39</v>
       </c>
-    </row>
-    <row r="26" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P25" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q25" s="10">
+        <v>52537899</v>
+      </c>
+    </row>
+    <row r="26" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E26" s="9" t="s">
         <v>15</v>
       </c>
@@ -7213,8 +7585,14 @@
       <c r="N26">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="27" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P26" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q26" s="10">
+        <v>61545441</v>
+      </c>
+    </row>
+    <row r="27" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E27" s="9" t="s">
         <v>56</v>
       </c>
@@ -7240,8 +7618,14 @@
       <c r="N27">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="28" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P27" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q27" s="10">
+        <v>1899624</v>
+      </c>
+    </row>
+    <row r="28" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E28" s="9" t="s">
         <v>54</v>
       </c>
@@ -7267,8 +7651,14 @@
       <c r="N28">
         <v>4.99</v>
       </c>
-    </row>
-    <row r="29" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P28" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q28" s="10">
+        <v>2368971</v>
+      </c>
+    </row>
+    <row r="29" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E29" s="9" t="s">
         <v>66</v>
       </c>
@@ -7294,8 +7684,14 @@
       <c r="N29">
         <v>4.99</v>
       </c>
-    </row>
-    <row r="30" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P29" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q29" s="10">
+        <v>529037</v>
+      </c>
+    </row>
+    <row r="30" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E30" s="9" t="s">
         <v>58</v>
       </c>
@@ -7321,8 +7717,14 @@
       <c r="N30">
         <v>2.09</v>
       </c>
-    </row>
-    <row r="31" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P30" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q30" s="10">
+        <v>1406861</v>
+      </c>
+    </row>
+    <row r="31" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E31" s="9" t="s">
         <v>33</v>
       </c>
@@ -7348,8 +7750,14 @@
       <c r="N31">
         <v>2.09</v>
       </c>
-    </row>
-    <row r="32" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P31" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q31" s="10">
+        <v>34951234</v>
+      </c>
+    </row>
+    <row r="32" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E32" s="9" t="s">
         <v>64</v>
       </c>
@@ -7375,8 +7783,14 @@
       <c r="N32">
         <v>0.56999999999999995</v>
       </c>
-    </row>
-    <row r="33" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P32" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q32" s="10">
+        <v>394341</v>
+      </c>
+    </row>
+    <row r="33" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E33" s="9" t="s">
         <v>41</v>
       </c>
@@ -7402,8 +7816,14 @@
       <c r="N33">
         <v>0.56999999999999995</v>
       </c>
-    </row>
-    <row r="34" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P33" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q33" s="10">
+        <v>17316800</v>
+      </c>
+    </row>
+    <row r="34" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E34" s="9" t="s">
         <v>27</v>
       </c>
@@ -7429,8 +7849,14 @@
       <c r="N34">
         <v>1.04</v>
       </c>
-    </row>
-    <row r="35" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P34" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q34" s="10">
+        <v>51540236</v>
+      </c>
+    </row>
+    <row r="35" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E35" s="9" t="s">
         <v>68</v>
       </c>
@@ -7456,8 +7882,14 @@
       <c r="N35">
         <v>1.04</v>
       </c>
-    </row>
-    <row r="36" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P35" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>455962</v>
+      </c>
+    </row>
+    <row r="36" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E36" s="9" t="s">
         <v>25</v>
       </c>
@@ -7483,8 +7915,14 @@
       <c r="N36">
         <v>2.72</v>
       </c>
-    </row>
-    <row r="37" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P36" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q36" s="10">
+        <v>37189229</v>
+      </c>
+    </row>
+    <row r="37" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E37" s="9" t="s">
         <v>52</v>
       </c>
@@ -7510,8 +7948,14 @@
       <c r="N37">
         <v>2.72</v>
       </c>
-    </row>
-    <row r="38" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P37" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q37" s="10">
+        <v>2710051</v>
+      </c>
+    </row>
+    <row r="38" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E38" s="9" t="s">
         <v>13</v>
       </c>
@@ -7537,8 +7981,14 @@
       <c r="N38">
         <v>5.05</v>
       </c>
-    </row>
-    <row r="39" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P38" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q38" s="10">
+        <v>155111022</v>
+      </c>
+    </row>
+    <row r="39" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E39" s="9" t="s">
         <v>48</v>
       </c>
@@ -7564,8 +8014,14 @@
       <c r="N39">
         <v>5.05</v>
       </c>
-    </row>
-    <row r="40" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P39" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q39" s="10">
+        <v>7025583</v>
+      </c>
+    </row>
+    <row r="40" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E40" s="9" t="s">
         <v>19</v>
       </c>
@@ -7582,8 +8038,14 @@
       <c r="N40">
         <v>2.76</v>
       </c>
-    </row>
-    <row r="41" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P40" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q40" s="10">
+        <v>62213676</v>
+      </c>
+    </row>
+    <row r="41" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E41" s="9" t="s">
         <v>89</v>
       </c>
@@ -7600,8 +8062,14 @@
       <c r="N41">
         <v>2.76</v>
       </c>
-    </row>
-    <row r="42" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="P41" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q41" s="10">
+        <v>833652994</v>
+      </c>
+    </row>
+    <row r="42" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M42" s="9" t="s">
         <v>76</v>
       </c>
@@ -7609,7 +8077,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="43" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M43" s="11" t="s">
         <v>77</v>
       </c>
@@ -7617,7 +8085,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="44" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M44" s="9" t="s">
         <v>23</v>
       </c>
@@ -7625,7 +8093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M45" s="11" t="s">
         <v>24</v>
       </c>
@@ -7633,7 +8101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M46" s="9" t="s">
         <v>15</v>
       </c>
@@ -7641,7 +8109,7 @@
         <v>9.2799999999999994</v>
       </c>
     </row>
-    <row r="47" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M47" s="11" t="s">
         <v>16</v>
       </c>
@@ -7649,7 +8117,7 @@
         <v>9.2799999999999994</v>
       </c>
     </row>
-    <row r="48" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="5:17" x14ac:dyDescent="0.3">
       <c r="M48" s="9" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
perform some excel fucntion
</commit_message>
<xml_diff>
--- a/population.csv.xlsx
+++ b/population.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Indian Population Data Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7702198-624F-4507-9079-0E8E6F0779C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76C048E-E36C-48F5-8E42-E2DFB7ACDCB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
   </bookViews>
   <sheets>
     <sheet name="population" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId4"/>
-    <pivotCache cacheId="3" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="97">
   <si>
     <t>Rank</t>
   </si>
@@ -494,7 +494,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -698,6 +698,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -874,7 +880,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -891,10 +897,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2797,7 +2805,418 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{62D21C4D-F7A7-4C69-9E5C-A505D3EFBF2C}" name="PivotTable5" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="M5:N76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="36">
+        <item x="31"/>
+        <item x="4"/>
+        <item x="26"/>
+        <item x="13"/>
+        <item x="2"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="9"/>
+        <item x="16"/>
+        <item x="20"/>
+        <item x="18"/>
+        <item x="12"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="34"/>
+        <item x="5"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="28"/>
+        <item x="24"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="30"/>
+        <item x="6"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="34">
+        <item x="20"/>
+        <item x="27"/>
+        <item x="8"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item x="31"/>
+        <item x="18"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="9"/>
+        <item x="28"/>
+        <item x="4"/>
+        <item x="22"/>
+        <item x="25"/>
+        <item x="7"/>
+        <item x="17"/>
+        <item x="32"/>
+        <item x="23"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="24"/>
+        <item x="2"/>
+        <item x="26"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="12"/>
+        <item x="21"/>
+        <item x="19"/>
+        <item x="30"/>
+        <item x="11"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="36">
+        <item x="34"/>
+        <item x="33"/>
+        <item x="29"/>
+        <item x="27"/>
+        <item x="32"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="21"/>
+        <item x="24"/>
+        <item x="28"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="14"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="26"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="6"/>
+        <item x="15"/>
+        <item x="10"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="18"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="34">
+        <item x="24"/>
+        <item x="29"/>
+        <item x="26"/>
+        <item x="17"/>
+        <item x="28"/>
+        <item x="22"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="20"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="12"/>
+        <item x="11"/>
+        <item x="13"/>
+        <item x="6"/>
+        <item x="15"/>
+        <item x="30"/>
+        <item x="0"/>
+        <item x="10"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="25"/>
+        <item x="27"/>
+        <item x="16"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="71">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i r="1">
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i r="1">
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i r="1">
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i r="1">
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i r="1">
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i r="1">
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i r="1">
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i r="1">
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i r="1">
+      <x v="20"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="11" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Sum of % of Total Population" fld="4" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{62D21C4D-F7A7-4C69-9E5C-A505D3EFBF2C}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="P5:Q41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -3027,8 +3446,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:K39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -3296,8 +3715,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:G41" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0">
@@ -3767,7 +4186,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{80C3E7D3-975D-432E-ACA4-EC6B906FDDBE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
@@ -3938,417 +4357,6 @@
   </pageFields>
   <dataFields count="1">
     <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="M5:N76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="36">
-        <item x="31"/>
-        <item x="4"/>
-        <item x="26"/>
-        <item x="13"/>
-        <item x="2"/>
-        <item x="29"/>
-        <item x="15"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="17"/>
-        <item x="25"/>
-        <item x="9"/>
-        <item x="16"/>
-        <item x="20"/>
-        <item x="18"/>
-        <item x="12"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="34"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="23"/>
-        <item x="22"/>
-        <item x="28"/>
-        <item x="24"/>
-        <item x="10"/>
-        <item x="27"/>
-        <item x="14"/>
-        <item x="7"/>
-        <item x="30"/>
-        <item x="6"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="19"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="34">
-        <item x="20"/>
-        <item x="27"/>
-        <item x="8"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item x="31"/>
-        <item x="18"/>
-        <item x="16"/>
-        <item x="13"/>
-        <item x="9"/>
-        <item x="28"/>
-        <item x="4"/>
-        <item x="22"/>
-        <item x="25"/>
-        <item x="7"/>
-        <item x="17"/>
-        <item x="32"/>
-        <item x="23"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="24"/>
-        <item x="2"/>
-        <item x="26"/>
-        <item x="29"/>
-        <item x="15"/>
-        <item x="12"/>
-        <item x="21"/>
-        <item x="19"/>
-        <item x="30"/>
-        <item x="11"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="36">
-        <item x="34"/>
-        <item x="33"/>
-        <item x="29"/>
-        <item x="27"/>
-        <item x="32"/>
-        <item x="17"/>
-        <item x="25"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="21"/>
-        <item x="24"/>
-        <item x="28"/>
-        <item x="23"/>
-        <item x="22"/>
-        <item x="11"/>
-        <item x="16"/>
-        <item x="14"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="13"/>
-        <item x="12"/>
-        <item x="26"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="6"/>
-        <item x="15"/>
-        <item x="10"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="18"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="34">
-        <item x="24"/>
-        <item x="29"/>
-        <item x="26"/>
-        <item x="17"/>
-        <item x="28"/>
-        <item x="22"/>
-        <item x="21"/>
-        <item x="18"/>
-        <item x="20"/>
-        <item x="14"/>
-        <item x="7"/>
-        <item x="5"/>
-        <item x="9"/>
-        <item x="4"/>
-        <item x="8"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="23"/>
-        <item x="12"/>
-        <item x="11"/>
-        <item x="13"/>
-        <item x="6"/>
-        <item x="15"/>
-        <item x="30"/>
-        <item x="0"/>
-        <item x="10"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="32"/>
-        <item x="31"/>
-        <item x="25"/>
-        <item x="27"/>
-        <item x="16"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="1"/>
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="71">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i r="1">
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i r="1">
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i r="1">
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i r="1">
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i r="1">
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i r="1">
-      <x v="20"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="11" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Sum of % of Total Population" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -6289,9 +6297,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F431FBD6-011F-415B-9936-0AA40F6E0697}">
-  <dimension ref="A2:X9"/>
+  <dimension ref="A2:X14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
@@ -6308,19 +6317,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="E2" s="13" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="E2" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="13"/>
-      <c r="H2" s="13" t="s">
+      <c r="F2" s="14"/>
+      <c r="H2" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="13"/>
+      <c r="I2" s="14"/>
       <c r="L2" s="7" t="s">
         <v>1</v>
       </c>
@@ -6362,22 +6371,22 @@
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="12">
+      <c r="A3" s="15">
         <f>MAX(population!E2:E36)</f>
         <v>16.5</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="E3" s="12">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="E3" s="15">
         <f>MAX(population!H2:H36)</f>
         <v>1084</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="H3" s="12">
+      <c r="F3" s="15"/>
+      <c r="H3" s="15">
         <f>MAX(population!I2:I36)</f>
         <v>94</v>
       </c>
-      <c r="I3" s="12"/>
+      <c r="I3" s="15"/>
       <c r="L3" s="6" t="s">
         <v>13</v>
       </c>
@@ -6462,19 +6471,19 @@
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="E5" s="13" t="s">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="E5" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="13"/>
-      <c r="H5" s="13" t="s">
+      <c r="F5" s="14"/>
+      <c r="H5" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="13"/>
+      <c r="I5" s="14"/>
       <c r="L5" s="6" t="s">
         <v>54</v>
       </c>
@@ -6517,22 +6526,22 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
+      <c r="A6" s="15">
         <f>MIN(population!E2:E36)</f>
         <v>0.01</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="E6" s="12">
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="E6" s="15">
         <f>MIN(population!H2:H36)</f>
         <v>618</v>
       </c>
-      <c r="F6" s="12"/>
-      <c r="H6" s="12">
+      <c r="F6" s="15"/>
+      <c r="H6" s="15">
         <f>MIN(population!I2:I36)</f>
         <v>61.8</v>
       </c>
-      <c r="I6" s="12"/>
+      <c r="I6" s="15"/>
       <c r="L6" s="6" t="s">
         <v>68</v>
       </c>
@@ -6617,19 +6626,19 @@
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="E8" s="13" t="s">
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="E8" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="F8" s="13"/>
-      <c r="H8" s="13" t="s">
+      <c r="F8" s="14"/>
+      <c r="H8" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="13"/>
+      <c r="I8" s="14"/>
       <c r="L8" s="6" t="s">
         <v>62</v>
       </c>
@@ -6672,22 +6681,22 @@
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="12">
+      <c r="A9" s="15">
         <f>AVERAGE(population!E2:E36)</f>
         <v>2.8568571428571428</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="E9" s="12">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="E9" s="15">
         <f>AVERAGE(population!H2:H36)</f>
         <v>931.2285714285714</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="H9" s="12">
+      <c r="F9" s="15"/>
+      <c r="H9" s="15">
         <f>AVERAGE(population!I11)</f>
         <v>78.03</v>
       </c>
-      <c r="I9" s="12"/>
+      <c r="I9" s="15"/>
       <c r="L9" s="6" t="s">
         <v>66</v>
       </c>
@@ -6729,14 +6738,25 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="12">
+        <f>VLOOKUP(A14,population!B2:N36,3,FALSE)</f>
+        <v>2966889</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A8:C8"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
@@ -6749,6 +6769,12 @@
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H8:I8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>